<commit_message>
Configura PWA instalável para Android e iOS
</commit_message>
<xml_diff>
--- a/public/modelo-aceitabilidade-creches.xlsx
+++ b/public/modelo-aceitabilidade-creches.xlsx
@@ -1238,6 +1238,52 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>5</col>
+      <colOff>619125</colOff>
+      <row>0</row>
+      <rowOff>9525</rowOff>
+    </from>
+    <to>
+      <col>5</col>
+      <colOff>1755140</colOff>
+      <row>5</row>
+      <rowOff>3810</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Imagem 1" descr="Logo Alimentação"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="11146155" y="9525"/>
+          <a:ext cx="1136015" cy="994410"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -2293,5 +2339,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="22" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>